<commit_message>
Update toolchain version 4.2.4
</commit_message>
<xml_diff>
--- a/compiler-ext.xlsx
+++ b/compiler-ext.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\issuehsu\work\gen-compiler-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAC9AC31-2E9E-4937-ACCA-DE3381734F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A78906-B198-4B4E-A253-D9CBB07E319B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,10 +60,10 @@
     <t>clang-4.1.0</t>
   </si>
   <si>
-    <t>gcc-4.2.3</t>
-  </si>
-  <si>
-    <t>clang-4.2.3</t>
+    <t>gcc-4.2.4</t>
+  </si>
+  <si>
+    <t>clang-4.2.4</t>
   </si>
   <si>
     <t>a</t>

</xml_diff>